<commit_message>
pasado a latex sin formato usach
</commit_message>
<xml_diff>
--- a/catedra/material/unidades/02-etica/Actividad-1/Inscirpcion/Actividad 1 (Ética en Investigación - Rol del Investigador) - Inscripción.xlsx
+++ b/catedra/material/unidades/02-etica/Actividad-1/Inscirpcion/Actividad 1 (Ética en Investigación - Rol del Investigador) - Inscripción.xlsx
@@ -13,13 +13,13 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={5a7a479a-8e76-4225-8eaf-2033830a51ec}</author>
-    <author>tc={8723d5af-df00-4e4e-b040-cae298f74616}</author>
-    <author>tc={cae6da80-0832-4355-b366-4b41c2c9104e}</author>
-    <author>tc={f8fc6f3e-108f-41c0-9703-4b4cd961278f}</author>
+    <author>tc={3359ac1c-afc3-4caa-8565-714de50aaac0}</author>
+    <author>tc={573e138d-c5f5-4aed-9e01-9254c5bac569}</author>
+    <author>tc={cd68a7d3-2da8-42b9-9759-4723748fe4fd}</author>
+    <author>tc={e71af6f3-e65b-41ec-bcd5-95b19394053d}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{5a7a479a-8e76-4225-8eaf-2033830a51ec}" ref="A7">
+    <comment authorId="0" xr:uid="{3359ac1c-afc3-4caa-8565-714de50aaac0}" ref="A7">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -28,7 +28,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{8723d5af-df00-4e4e-b040-cae298f74616}" ref="C8">
+    <comment authorId="1" xr:uid="{573e138d-c5f5-4aed-9e01-9254c5bac569}" ref="C8">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -37,16 +37,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{cae6da80-0832-4355-b366-4b41c2c9104e}" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Ioan Mang tiene varios casos de plagio, nos centraremos en otro distinto de ustedes
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{f8fc6f3e-108f-41c0-9703-4b4cd961278f}" ref="A1">
+    <comment authorId="2" xr:uid="{cd68a7d3-2da8-42b9-9759-4723748fe4fd}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -57,12 +48,24 @@
 </t>
       </text>
     </comment>
+    <comment authorId="3" xr:uid="{e71af6f3-e65b-41ec-bcd5-95b19394053d}" ref="A1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Ioan Mang tiene varios casos de plagio, nos centraremos en otro distinto de ustedes
+</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+  <si>
+    <t>Fecha Actividad: 09/09/2026</t>
+  </si>
   <si>
     <t xml:space="preserve"> Los casos no se pueden repetir. Indique nombre del caso y autores involucrados</t>
   </si>
@@ -70,7 +73,7 @@
     <t>USO INTERNO</t>
   </si>
   <si>
-    <t>Estudiante</t>
+    <t>Grupo</t>
   </si>
   <si>
     <t>Orden de presentación
@@ -83,116 +86,35 @@
     <t>Caso 2 (Informática)</t>
   </si>
   <si>
-    <t>Jonathan Valenzuela</t>
+    <t>Grupo 1</t>
   </si>
   <si>
-    <t>Karl-Theodor zu Guttenberg - Plagio de Tesis Doctoral (Derecho</t>
+    <t>Caso Jan Hendrik Schön (Física / Nanotecnología, Bell Labs, EE. UU. / Univ. de Konstanz, Alemania). Publicaciones en Science, Nature y Appl. Phys. Lett. Schön fabricó y falsificó sistemáticamente datos sobre superconductividad y transistores moleculares, reutilizando curvas y gráficos idénticos para experimentos distintos y destruyendo los datos primarios.</t>
   </si>
   <si>
-    <t>Chen-Yuan Chen - Anillo de Revisión por Pares (Peer-Review Ring) en 2014</t>
+    <t>Escándalo de Retracciones Masivas de ACM (Ciencias de la Computación / Inteligencia Artificial). Conferencias ACM ICICN y ICISS (2021-2022), denunciado por G. Cabanac, C. Labbé y A. Magazinov. Se evidenció la operación de fábricas de artículos (paper mills), manipulación de revisión por pares y uso de parafraseo algorítmico ("tortured phrases") para evadir el plagio en actas de congresos de computación. Culminó con la retractación de más de 320 artículos por parte de la ACM y la reforma integral de su sistema de integridad científica.</t>
   </si>
   <si>
-    <t>Alejandro Jesús Pirez Prendes</t>
+    <t>Grupo 4</t>
   </si>
   <si>
-    <t>Jan Hendrik Schön (Bell Labs) y 20 coautores exonerados - Fraude Schön en Bell Labs -  Fabricación de datos en física de materiales (superconductividad, electrónica molecular). Retractación de &gt;15 artículos en Science y Nature (2002-2003).</t>
+    <t>Caso de Victor Ninov y el falso descubrimiento del elemento 118. En 1999, un equipo del Lawrence Berkeley National Laboratory publicó en Physical Review Letters el supuesto descubrimiento del elemento 118 a partir de señales de desintegración nuclear. Tras múltiples intentos fallidos de reproducir los resultados, una investigación interna concluyó que datos fundamentales habían sido fabricados, atribuyéndose la mala conducta científica al investigador Victor Ninov. El artículo fue posteriormente retractado.</t>
   </si>
   <si>
-    <t xml:space="preserve">Shadi Aljawarneh (JUST), V. Radhakrishna, A. Cheruvu - Falsificación de citas en ACM - Manipulación de referencias para inflar artificialmente las citas y el índice h. Retractación de 27 artículos por la ACM en 2025.        </t>
+    <t>Grupo 3</t>
   </si>
   <si>
-    <t>Pier Miqueles</t>
+    <t>El Caso Bengü Sezen: El falso "Milagro" de la Síntesis QuímicaA principios de la década de 2000, la estudiante de doctorado Bengü Sezen trabajaba en el laboratorio de química del respetado profesor Dalibor Sames en la Universidad de Columbia. [1] (https://cen.acs.org/articles/89/i32/Puzzle-Named-BengSezen.html), [2] (https://www.enago.com/academy/research-misconduct-bengu-sezen-case/)El supuesto avance: Sezen afirmó haber descubierto un método revolucionario para la activación de enlaces C-H (carbono-hidrógeno). Este proceso es uno de los "Santos Griales" de la química orgánica, ya que permite modificar hidrocarburos de forma selectiva para crear medicamentos o materiales complejos de manera mucho más rápida y barata</t>
   </si>
   <si>
-    <t>Jesús Ángel Lemus. (Inventaba resultados de análisis de laboratorio que nunca ocurrieron.)</t>
-  </si>
-  <si>
-    <t>Alexander Spivak (Plagio y Falsificación en IA)</t>
-  </si>
-  <si>
-    <t>Joel Fuertes</t>
-  </si>
-  <si>
-    <t>El caso de las células STAP: falsificación y plagio en publicaciones de biología celular</t>
-  </si>
-  <si>
-    <t>El caso de Juan Manuel Corchado: Manipulación sistemática de citas en informática</t>
-  </si>
-  <si>
-    <t>Javier Gomez</t>
-  </si>
-  <si>
-    <t>Thereza Imanishi-Kari , David Baltimore - El escándalo de falsificación de datos en el MIT</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="0"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Shahaboddin Shamshirband Dalibor Petković</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> - </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="0"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>El Escándalo de Shahaboddin Shamshirband</t>
-    </r>
-  </si>
-  <si>
-    <t>Casos de Experimentacion con seres humanos</t>
-  </si>
-  <si>
-    <t>CASO HISTÓRICO – "CONEJILLOS DE INDIAS": LA EXPERIMENTACIÓN QUÍMICA EN PRISIONEROS POLÍTICOS CHILENOS (1981)</t>
-  </si>
-  <si>
-    <t>CASO EN INFORMÁTICA – NEUROTECNOLOGÍA Y DERECHOS HUMANOS: EL CASO GIRARDI VS. EMOTIV INC.</t>
-  </si>
-  <si>
-    <t>Alejandro Pirez</t>
-  </si>
-  <si>
-    <t>Experimentos de Aplastamiento de Columna Vertebral en Conejos en el Instituto Karolinska</t>
-  </si>
-  <si>
-    <t>Manipulación mediante Inteligencia Artificial sin Consentimiento en Reddit</t>
-  </si>
-  <si>
-    <t>Jonatahn Valenzuela</t>
-  </si>
-  <si>
-    <t>Hwang Woo-suk. - El Fraude de la clonación</t>
-  </si>
-  <si>
-    <t>Lorenza Colzato - Neurociencia e Informática Cognitiva</t>
-  </si>
-  <si>
-    <t>Caso histórico: Experimento del “Pequeño Albert”</t>
-  </si>
-  <si>
-    <t>El conjunto de datos de OKCupid: publicación de datos 
-personales de usuarios de una plataforma de citas</t>
-  </si>
-  <si>
-    <t>Biopsias musculares en estudiantes – Universidad Finis Terrae  (Hermann Zbinden)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experimento de contagio emocional en Facebook (Adam D. I. Kramer) </t>
+    <t>Caso de Chen-Yuan Chen (Informática y Algoritmos, National Pingtung University of Education, Taiwán). Fraude por manipulación del sistema de revisión (FFP/QRP). Chen creó más de 130 cuentas de correo electrónico con identidades falsas o asumidas para actuar como revisor anónimo de sus propios artículos científicos. Tras una extensa investigación, la revista Journal of Vibration and Control (SAGE) retractó mas de 50 de sus publicaciones simultáneamente en 2014.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -213,15 +135,11 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="10.0"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="10.0"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
     </font>
     <font>
       <b/>
@@ -254,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -274,10 +192,10 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" vertical="center"/>
@@ -313,15 +231,12 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -342,25 +257,25 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Roberto Gonzalez Ibanez" id="{af7e0948-942b-4611-a953-6d3fa7cf2251}" providerId="google-sheets"/>
-  <x18tc:person displayName="Boris Bustos Valdebenito" id="{ae8fa3e4-2226-4473-98e6-6f22b1f9371b}" providerId="google-sheets"/>
-  <x18tc:person displayName="Alex Valentín Espinosa Rivera" id="{cecb5a3f-725a-45d6-b8ef-662750982d35}" providerId="google-sheets"/>
-  <x18tc:person displayName="Javier Valerio Morales" id="{81ca9794-fe2e-4dc6-ab60-9b2eff7f9f83}" providerId="google-sheets"/>
+  <x18tc:person displayName="Roberto Gonzalez Ibanez" id="{ee2ff593-f158-4ee3-b31a-379d6ddbda3c}" providerId="google-sheets"/>
+  <x18tc:person displayName="Boris Bustos Valdebenito" id="{3a01f83b-77de-4d09-941b-160dcd61088f}" providerId="google-sheets"/>
+  <x18tc:person displayName="Alex Valentín Espinosa Rivera" id="{986ec8d9-3383-4c07-9450-b86acc303634}" providerId="google-sheets"/>
+  <x18tc:person displayName="Javier Valerio Morales" id="{d8628ed5-9e68-4668-afee-8328a3a9f65f}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2021-09-14T22:26:43.00" personId="{81ca9794-fe2e-4dc6-ab60-9b2eff7f9f83}" id="{cae6da80-0832-4355-b366-4b41c2c9104e}" done="1">
+  <x18tc:threadedComment ref="A1" dT="2021-09-14T22:26:43.00" personId="{d8628ed5-9e68-4668-afee-8328a3a9f65f}" id="{e71af6f3-e65b-41ec-bcd5-95b19394053d}" done="1">
     <x18tc:text xml:space="preserve">Ioan Mang tiene varios casos de plagio, nos centraremos en otro distinto de ustedes</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2021-09-09T23:41:02.00" personId="{af7e0948-942b-4611-a953-6d3fa7cf2251}" id="{f8fc6f3e-108f-41c0-9703-4b4cd961278f}" done="1">
+  <x18tc:threadedComment ref="A1" dT="2021-09-09T23:41:02.00" personId="{ee2ff593-f158-4ee3-b31a-379d6ddbda3c}" id="{cd68a7d3-2da8-42b9-9759-4723748fe4fd}" done="1">
     <x18tc:text xml:space="preserve">Cuidado, podría no ajustarse a lo que se considera un caso válido para el curso (al menos basado en la información indicada). Pues se trata de casos de falta a la ética en investigación/investigación aplicada</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2021-09-15T00:00:33.00" personId="{ae8fa3e4-2226-4473-98e6-6f22b1f9371b}" id="{c272f25f-405e-44ce-b83b-b550d0296fc1}" parentId="{f8fc6f3e-108f-41c0-9703-4b4cd961278f}">
+  <x18tc:threadedComment ref="A1" dT="2021-09-15T00:00:33.00" personId="{3a01f83b-77de-4d09-941b-160dcd61088f}" id="{e3746cf2-3cd5-4342-93c0-33415de19a3c}" parentId="{cd68a7d3-2da8-42b9-9759-4723748fe4fd}">
     <x18tc:text xml:space="preserve">Tema modificado</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A7" dT="2022-09-09T01:22:59.00" personId="{cecb5a3f-725a-45d6-b8ef-662750982d35}" id="{5a7a479a-8e76-4225-8eaf-2033830a51ec}" done="1">
+  <x18tc:threadedComment ref="A7" dT="2022-09-09T01:22:59.00" personId="{986ec8d9-3383-4c07-9450-b86acc303634}" id="{3359ac1c-afc3-4caa-8565-714de50aaac0}" done="1">
     <x18tc:text xml:space="preserve">No tengo equipo, pero si a alguien le interesa los casos que dejé, estoy en telegram:  https://t.me/Alex_chama</x18tc:text>
     <x18tc:extLst>
       <ext uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -369,7 +284,7 @@
       </ext>
     </x18tc:extLst>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="C8" dT="2023-09-27T20:46:07.00" personId="{af7e0948-942b-4611-a953-6d3fa7cf2251}" id="{8723d5af-df00-4e4e-b040-cae298f74616}" done="1">
+  <x18tc:threadedComment ref="C8" dT="2023-09-27T20:46:07.00" personId="{ee2ff593-f158-4ee3-b31a-379d6ddbda3c}" id="{573e138d-c5f5-4aed-9e01-9254c5bac569}" done="1">
     <x18tc:text xml:space="preserve">Es una publicación?</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -385,19 +300,21 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="48.88"/>
     <col customWidth="1" min="2" max="2" width="24.5"/>
-    <col customWidth="1" min="3" max="3" width="55.0"/>
-    <col customWidth="1" min="4" max="4" width="163.0"/>
+    <col customWidth="1" min="3" max="3" width="71.13"/>
+    <col customWidth="1" min="4" max="4" width="55.88"/>
     <col customWidth="1" min="6" max="6" width="27.75"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -424,7 +341,7 @@
     <row r="2">
       <c r="A2" s="4"/>
       <c r="B2" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -452,16 +369,16 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -485,15 +402,15 @@
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
     </row>
-    <row r="4">
+    <row r="4" ht="53.25" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -518,16 +435,9 @@
       <c r="Y4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>9</v>
-      </c>
       <c r="B5" s="8"/>
-      <c r="C5" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="10"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -551,16 +461,10 @@
       <c r="Y5" s="3"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="s">
-        <v>12</v>
-      </c>
+      <c r="A6" s="11"/>
       <c r="B6" s="12"/>
-      <c r="C6" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>14</v>
-      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -585,15 +489,13 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B7" s="16"/>
       <c r="C7" s="17" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
-      <c r="D7" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D7" s="17"/>
       <c r="E7" s="18"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -616,16 +518,16 @@
       <c r="X7" s="3"/>
       <c r="Y7" s="3"/>
     </row>
-    <row r="8" ht="43.5" customHeight="1">
+    <row r="8" ht="92.25" customHeight="1">
       <c r="A8" s="18" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="19" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>20</v>
+      <c r="D8" s="18" t="s">
+        <v>14</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -677,10 +579,10 @@
       <c r="Y9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="21"/>
+      <c r="A10" s="20"/>
       <c r="B10" s="18"/>
       <c r="C10" s="18"/>
-      <c r="D10" s="21"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -706,9 +608,7 @@
     <row r="11">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
-      <c r="C11" s="22" t="s">
-        <v>21</v>
-      </c>
+      <c r="C11" s="21"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -733,16 +633,10 @@
       <c r="Y11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="s">
-        <v>18</v>
-      </c>
+      <c r="A12" s="18"/>
       <c r="B12" s="3"/>
-      <c r="C12" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>23</v>
-      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -766,16 +660,10 @@
       <c r="Y12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="s">
-        <v>24</v>
-      </c>
+      <c r="A13" s="18"/>
       <c r="B13" s="3"/>
-      <c r="C13" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>26</v>
-      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -799,16 +687,10 @@
       <c r="Y13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="s">
-        <v>27</v>
-      </c>
+      <c r="A14" s="18"/>
       <c r="B14" s="3"/>
-      <c r="C14" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>29</v>
-      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -832,16 +714,10 @@
       <c r="Y14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="s">
-        <v>15</v>
-      </c>
+      <c r="A15" s="18"/>
       <c r="B15" s="3"/>
-      <c r="C15" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>31</v>
-      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -865,16 +741,10 @@
       <c r="Y15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="s">
-        <v>12</v>
-      </c>
+      <c r="A16" s="18"/>
       <c r="B16" s="3"/>
-      <c r="C16" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>33</v>
-      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>

</xml_diff>